<commit_message>
feat: add multiple variables in single cell support
</commit_message>
<xml_diff>
--- a/o23-n6/test/template.xlsx
+++ b/o23-n6/test/template.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10503"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EF52A26-B878-E84F-8C1B-0BB109ABF89F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5504EA62-369B-7C48-9CCD-024D42D23546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -131,7 +131,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <si>
     <t>SUMMARY OF TOTAL COLLECTIONS - SGD</t>
   </si>
@@ -208,21 +208,23 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>$summary.field2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>$name</t>
+  </si>
+  <si>
+    <t>$.$del</t>
+  </si>
+  <si>
+    <t>$.num.subTotal.cashInTxn</t>
+  </si>
+  <si>
     <t>$summary.field1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>$summary.field2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>$name</t>
-  </si>
-  <si>
-    <t>$.$del</t>
-  </si>
-  <si>
-    <t>$.num.subTotal.cashInTxn</t>
+  </si>
+  <si>
+    <t>${summary.field1}, ${summary.field2}, $\{summary.field2}, ${summary.field2\}</t>
   </si>
 </sst>
 </file>
@@ -654,10 +656,10 @@
     </row>
     <row r="5" spans="1:5" ht="16">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>9</v>
@@ -671,13 +673,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
         <v>16</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>12</v>
@@ -708,10 +710,10 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C10" t="s">
         <v>13</v>
@@ -722,10 +724,13 @@
     </row>
     <row r="13" spans="1:5">
       <c r="B13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" t="s">
         <v>19</v>
       </c>
-      <c r="C13" t="s">
-        <v>20</v>
+      <c r="D13" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>